<commit_message>
fix: 2026-07-14 - misc fixes (#544)
* fix: initial misc fixes

* fix: second commit

* fix: third commit
</commit_message>
<xml_diff>
--- a/next/app/compliance-reporting/lib/model-year-reports/templates/assessment_template.xlsx
+++ b/next/app/compliance-reporting/lib/model-year-reports/templates/assessment_template.xlsx
@@ -1,27 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/timchen/Desktop/zeva/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1916526C-CB57-764A-9AD0-9A16661C2187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDFE870F-200A-2441-BF7B-CC2296383B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2280" yWindow="2880" windowWidth="32280" windowHeight="16940" xr2:uid="{596842B5-1F9C-BB4A-9EA7-2707F0F20405}"/>
   </bookViews>
   <sheets>
     <sheet name="Details" sheetId="1" r:id="rId1"/>
     <sheet name="Compliance Ratio Reductions" sheetId="2" r:id="rId2"/>
-    <sheet name="Beginning Balance" sheetId="10" r:id="rId3"/>
-    <sheet name="Credits" sheetId="6" r:id="rId4"/>
-    <sheet name="Previous Adjustments" sheetId="7" r:id="rId5"/>
-    <sheet name="Current Adjustments" sheetId="9" r:id="rId6"/>
-    <sheet name="Offsets and Transfers Away" sheetId="5" r:id="rId7"/>
-    <sheet name="Final Ending Balance" sheetId="3" r:id="rId8"/>
-    <sheet name="Statement(s)" sheetId="4" r:id="rId9"/>
+    <sheet name="ZEV and ICE Counts" sheetId="11" r:id="rId3"/>
+    <sheet name="Beginning Balance" sheetId="10" r:id="rId4"/>
+    <sheet name="Credits" sheetId="6" r:id="rId5"/>
+    <sheet name="Previous Adjustments" sheetId="7" r:id="rId6"/>
+    <sheet name="Current Adjustments" sheetId="9" r:id="rId7"/>
+    <sheet name="Offsets and Transfers Away" sheetId="5" r:id="rId8"/>
+    <sheet name="Final Ending Balance" sheetId="3" r:id="rId9"/>
+    <sheet name="Statement(s)" sheetId="4" r:id="rId10"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="17">
   <si>
     <t>Model Year</t>
   </si>
@@ -88,6 +89,12 @@
   </si>
   <si>
     <t>Compliant</t>
+  </si>
+  <si>
+    <t>ZEV Count</t>
+  </si>
+  <si>
+    <t>ICE Count</t>
   </si>
 </sst>
 </file>
@@ -492,6 +499,18 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A603B588-451E-DE47-B4C5-80CCA31AA744}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="135.5" customWidth="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A228C30-8AB9-C445-9148-E3AA65C63F60}">
   <dimension ref="A1:F1"/>
@@ -530,6 +549,32 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DA58B50-B889-1446-9F7E-5EE3B5BBD16A}">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="20.5" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70438796-C504-964A-BE49-E27234E80981}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -563,7 +608,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{092B32A8-1A64-2347-99F3-32905DDC8385}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -596,7 +641,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B63D4D29-49CB-FE47-AAC8-5E814C359DDB}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -630,7 +675,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06F2F3A0-C836-3C4C-9B76-FCF87CCE7131}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -664,7 +709,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{240610B3-BA6F-EA4D-8E64-BC14F2315C65}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -698,7 +743,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59281AEA-3AA5-0C4E-A67E-4D6171492622}">
   <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -736,16 +781,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A603B588-451E-DE47-B4C5-80CCA31AA744}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="135.5" customWidth="1"/>
-  </cols>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>